<commit_message>
Add application API test cases
</commit_message>
<xml_diff>
--- a/acquiring_api_attachment_test_cases.xlsx
+++ b/acquiring_api_attachment_test_cases.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Attachment tests" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Application tests" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Attachment tests'!$A$1:$F$11</definedName>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="118">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -194,6 +195,189 @@
   </si>
   <si>
     <t xml:space="preserve">500 Internal Server Error; код ошибки ATTACHMENT_METADATA_SAVE_ERROR; загруженный файл удаляется, запись метаданных не создаётся.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Название </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тестовые данные</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Приоритет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Успешное создание заявки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API запущен, PostgreSQL доступен </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отправить POST /applications с корректным JSON и новым Idempotency-Key </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Корректные ФИО, телефон, ИНН, source=SITE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">201 Created; возвращены applicationId, status=NEW, innVerificationStatus=PENDING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отсутствует Idempotency-Key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API запущен</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отправить POST /applications без заголовка Idempotency-Key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Корректное тело заявки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">400 VALIDATION_ERROR; заявка не создаётся</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Повтор с тем же ключом и данными</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Заявка уже создана</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Повторить POST /applications с тем же ключом и тем же JSON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idempotency-Key и тело первого запроса</t>
+  </si>
+  <si>
+    <t xml:space="preserve">201 Created; возвращается тот же applicationId; дубликат не создаётся</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Повтор с тем же ключом и другими данными</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ключ уже использован</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Повторить POST /applications с тем же ключом, изменив одно поле</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тот же ключ, другое значение city</t>
+  </si>
+  <si>
+    <t xml:space="preserve">409 IDEMPOTENCY_KEY_REUSED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Некорректный телефон</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отправить POST /applications с некорректным phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">phone=12345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Некорректный формат ИНН </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> API запущен</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отправить POST /applications с ИНН неправильной длины</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inn=12345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Недопустимый источник заявки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отправить POST /applications с source, отсутствующим в enum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source=WEB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Проверка сохранения заявки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Заявка успешно создана</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выполнить SELECT по applicationId в PostgreSQL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">applicationId из ответа API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В БД существует одна соответствующая запись</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-09 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пустое значение телефона </t>
+  </si>
+  <si>
+    <t xml:space="preserve">API запущен </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отправить POST /applications с пустым phone и новым ключом </t>
+  </si>
+  <si>
+    <t xml:space="preserve">phone="" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">400 VALIDATION_ERROR; заявка не создаётся </t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP-10 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Повторный запрос после перезапуска API </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Заявка ранее создана и сохранена в PostgreSQL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Перезапустить API и повторить запрос с тем же ключом и тем же JSON </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ключ и тело ранее созданного запроса </t>
+  </si>
+  <si>
+    <t xml:space="preserve">201 Created; возвращается прежний applicationId </t>
   </si>
 </sst>
 </file>
@@ -203,7 +387,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -243,6 +427,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="2">
@@ -294,8 +485,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -303,7 +498,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -311,12 +506,24 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -360,230 +567,230 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="4" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="4" t="s">
         <v>56</v>
       </c>
     </row>
@@ -598,4 +805,284 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="31.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.03"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="58.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="46.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="46.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="36.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Обычный"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12&amp;KffffffСтраница &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Record application test results
</commit_message>
<xml_diff>
--- a/acquiring_api_attachment_test_cases.xlsx
+++ b/acquiring_api_attachment_test_cases.xlsx
@@ -377,7 +377,7 @@
     <t xml:space="preserve">Ключ и тело ранее созданного запроса </t>
   </si>
   <si>
-    <t xml:space="preserve">201 Created; возвращается прежний applicationId </t>
+    <t xml:space="preserve">201 Created, applicationId совпадает с результатом до перезапуска API</t>
   </si>
 </sst>
 </file>
@@ -510,19 +510,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -815,12 +815,12 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="31.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="31.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="23.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Update attachment test results
</commit_message>
<xml_diff>
--- a/acquiring_api_attachment_test_cases.xlsx
+++ b/acquiring_api_attachment_test_cases.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Attachment tests" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="149">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -44,6 +44,12 @@
     <t xml:space="preserve">Ожидаемый результат</t>
   </si>
   <si>
+    <t xml:space="preserve">Фактический результат </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Статус </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-001</t>
   </si>
   <si>
@@ -62,6 +68,12 @@
     <t xml:space="preserve">201 Created; в ответе есть attachmentId; файл сохранён и доступен для дальнейшей проверки ИНН.</t>
   </si>
   <si>
+    <t xml:space="preserve">201 Created — файл загружен </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-002</t>
   </si>
   <si>
@@ -77,6 +89,9 @@
     <t xml:space="preserve">201 Created; возвращён attachmentId; файл сохранён.</t>
   </si>
   <si>
+    <t xml:space="preserve">201 Created, файл успешно загружен. Для текущей проверки загружен PNG размером 2 567 746 байт</t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-003</t>
   </si>
   <si>
@@ -92,6 +107,9 @@
     <t xml:space="preserve"> 413 Content Too Large; файл не сохраняется как доступное вложение.</t>
   </si>
   <si>
+    <t xml:space="preserve">413 FILE_TOO_LARGE </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-004</t>
   </si>
   <si>
@@ -107,6 +125,9 @@
     <t xml:space="preserve">415 Unsupported Media Type; файл не сохранён как допустимый документ.</t>
   </si>
   <si>
+    <t xml:space="preserve">415 UNSUPPORTED_FILE_TYPE </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-005</t>
   </si>
   <si>
@@ -122,6 +143,9 @@
     <t xml:space="preserve">400 Bad Request; код ошибки, например EMPTY_FILE; attachmentId не выдаётся.</t>
   </si>
   <si>
+    <t xml:space="preserve">400 EMPTY_FILE </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-006</t>
   </si>
   <si>
@@ -134,6 +158,9 @@
     <t xml:space="preserve">400 Bad Request; код ошибки INVALID_FILE_CONTENT; загруженный файл удалён, запись вложения в БД не создаётся.</t>
   </si>
   <si>
+    <t xml:space="preserve">400 INVALID_FILE_CONTENT </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-007</t>
   </si>
   <si>
@@ -149,6 +176,12 @@
     <t xml:space="preserve">422 Unprocessable Content; файл отклонён или помещён в карантин и не может быть использован для подтверждения ИНН.</t>
   </si>
   <si>
+    <t xml:space="preserve">Проверка антивирусом не реализована; проверяется только сигнатура файла </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не реализован </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-008</t>
   </si>
   <si>
@@ -164,6 +197,9 @@
     <t xml:space="preserve">401 Unauthorized; файл не становится доступным.</t>
   </si>
   <si>
+    <t xml:space="preserve">Авторизация не реализована; ответ 401 не проверен </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-009</t>
   </si>
   <si>
@@ -179,6 +215,9 @@
     <t xml:space="preserve">403 Forbidden; файл не становится доступным.</t>
   </si>
   <si>
+    <t xml:space="preserve">Проверка прав доступа не реализована; ответ 403 не проверен </t>
+  </si>
+  <si>
     <t xml:space="preserve">ATT-010</t>
   </si>
   <si>
@@ -197,6 +236,48 @@
     <t xml:space="preserve">500 Internal Server Error; код ошибки ATTACHMENT_METADATA_SAVE_ERROR; загруженный файл удаляется, запись метаданных не создаётся.</t>
   </si>
   <si>
+    <t xml:space="preserve">Ожидаемая обработка ошибки — 500 ATTACHMENT_METADATA_SAVE_ERROR, с удалением уже сохранённого файла. Фактический запуск именно этого сценария в доступной истории не подтверждён </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не подтверждён </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATT-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Проверка сохранения файла на диске и метаданных в PostgreSQL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API запущен; PostgreSQL доступен; существует корректный PNG-файл размером менее 10 МБ; известна папка uploads текущего проекта. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Загрузить PNG через POST /attachments. Проверить наличие файла в uploads и выполнить SELECT из таблицы attachments по attachment_id. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Файл существует на диске. В БД есть запись с соответствующими attachment_id, file_path и file_size. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">201 Created; файл найден на диске, запись найдена в БД, attachment_id, путь и размер совпадают </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATT-012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Успешное скачивание вложения </t>
+  </si>
+  <si>
+    <t xml:space="preserve">API запущен; PostgreSQL доступен; вложение ранее успешно загружено через POST /attachments; файл существует на диске, а его метаданные сохранены в PostgreSQL; известен attachment_id. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выполнить GET /attachments/{attachment_id}/download для существующего вложения. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ответ 200 OK; скачанный файл совпадает с оригиналом по SHA256. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 OK; файл скачан; SHA256 совпадает с оригиналом </t>
+  </si>
+  <si>
     <t xml:space="preserve">Название </t>
   </si>
   <si>
@@ -293,6 +374,12 @@
     <t xml:space="preserve">phone=12345</t>
   </si>
   <si>
+    <t xml:space="preserve">400 — VALIDATION_ERROR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS</t>
+  </si>
+  <si>
     <t xml:space="preserve">APP-06</t>
   </si>
   <si>
@@ -341,6 +428,9 @@
     <t xml:space="preserve">В БД существует одна соответствующая запись</t>
   </si>
   <si>
+    <t xml:space="preserve">SELECT вернул 4 заявки; записи сохранены в PostgreSQL, статусы NEW и PENDING. </t>
+  </si>
+  <si>
     <t xml:space="preserve">APP-09 </t>
   </si>
   <si>
@@ -375,6 +465,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ключ и тело ранее созданного запроса </t>
+  </si>
+  <si>
+    <t xml:space="preserve">201 Created; возвращается прежний applicationId</t>
   </si>
   <si>
     <t xml:space="preserve">201 Created, applicationId совпадает с результатом до перезапуска API</t>
@@ -485,7 +578,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -502,14 +595,26 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -518,8 +623,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -564,14 +681,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="47.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -593,205 +713,323 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="42.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>8</v>
+      </c>
       <c r="B2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="G2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="H2" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="48.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G3" s="6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="H3" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="39.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="G4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="H4" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="50" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="B5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="G5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="H5" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="37.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="B6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="G6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="H6" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="40.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="B7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="G7" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="H7" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="43.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="G8" s="6" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="H8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="4" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="46.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="B9" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F9" s="5" t="s">
         <v>56</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="51.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="50" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -812,7 +1050,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.3"/>
@@ -821,259 +1059,316 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="23.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="21"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C1" s="6" t="s">
+      <c r="B1" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F1" s="7" t="s">
+      <c r="E1" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="58.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>66</v>
+      <c r="G1" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="H2" s="14"/>
+      <c r="I2" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="H3" s="14"/>
+      <c r="I3" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="H4" s="14"/>
+      <c r="I4" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="H5" s="14"/>
+      <c r="I5" s="7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="46.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>66</v>
+      <c r="A6" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="E7" s="8" t="s">
+      <c r="A7" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="H7" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="36.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+      <c r="D8" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="F8" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>111</v>
+      <c r="G8" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="I10" s="7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="47.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" s="8" t="s">
+      <c r="A11" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="I11" s="14" t="s">
         <v>117</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>